<commit_message>
Wheel list: motor already owned, keep the quick release
The hoverboard motor is already owned, so it drops to AUD 0. That frees
enough budget to keep DAZ's Arca-Swiss quick release (his cheaper option),
which is how the V2 base attaches to the desk. The wireless buttons and
paddles stay an optional upgrade. Wheel total is now about AUD 189.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QEYLvGWigrKvVwvVek2yBU
</commit_message>
<xml_diff>
--- a/parts-lists/DAZ_racing_V2_steering_wheel_budget_parts_list_AUD.xlsx
+++ b/parts-lists/DAZ_racing_V2_steering_wheel_budget_parts_list_AUD.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="162">
   <si>
     <t xml:space="preserve">DAZ Racing V2 Steering Wheel – budget parts list (AUD)</t>
   </si>
@@ -91,25 +91,19 @@
     <t xml:space="preserve">DAZ's link: €29.92 sale (May 2025) ≈ AUD 44 incl. GST. 2026 US-store listings US$37–41 ≈ AUD 59–65 incl. GST. Estimate AUD 50 (between the two – check the live price).</t>
   </si>
   <si>
-    <t xml:space="preserve">6.5" hoverboard motor – from a second-hand hoverboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 motor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Swapped – used hoverboard instead of a new motor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gumtree / Facebook Marketplace</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gumtree search: hoverboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Biggest single saving. A used or 'not working' hoverboard has two motors, and it's usually the battery or board that died, not the motors. Make sure the wheels are 6.5" (165 mm), spin freely and don't grind. Take the battery to a battery-recycling drop-off (e.g. B-cycle). Can't find one? A new motor through DAZ's link is ≈ AUD 40–50 delivered: https://s.click.aliexpress.com/e/_c3TEkURL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gumtree AU, 2026: working hoverboards from ≈ AUD 40–50; broken/for-parts ones cheaper or free. New 6.5" motor on AliExpress ≈ US$23–30 + shipping.</t>
+    <t xml:space="preserve">6.5" hoverboard motor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Already have – $0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You already own it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Before you print, check it's a 6.5" (165 mm) motor that spins freely and doesn't grind – DAZ's mount is sized for 6.5" motors.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You already have it, so it costs nothing.</t>
   </si>
   <si>
     <t xml:space="preserve">Rotary encoder E6B2-CWZ6C (6 mm shaft, NPN output)</t>
@@ -217,6 +211,27 @@
     <t xml:space="preserve">Typical 250 mm length US$2–3.50.</t>
   </si>
   <si>
+    <t xml:space="preserve">Quick-release clamp, Arca-Swiss (DAZ's cheaper 'option 2')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kept – DAZ's cheaper option</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is how DAZ's V2 base attaches to the desk (his "aluminum Quick-Release to detach from the desk"), so it's back in now that the motor costs nothing – the build goes together as designed. His first pick, a FANAUE lever clamp, is ≈ AUD 40+. This cheaper listing is titled as a plate: pick its clamp option if it has one; any Arca-Swiss clamp grips the 100 mm plate below.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cheap Arca-Swiss clamps US$5–11 (2026) ≈ AUD 8–17.50 incl. GST. Estimate AUD 16.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quick-release plate, Arca-Swiss, 100 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Goes with the clamp above.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typical listing US$3–5 ≈ AUD 4.80–7.90 incl. GST.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Subtotal – parts</t>
   </si>
   <si>
@@ -328,31 +343,16 @@
     <t xml:space="preserve">TOTAL – counts toward the AUD budget</t>
   </si>
   <si>
-    <t xml:space="preserve">4. REMOVED TO STAY UNDER BUDGET – optional add-ons (NOT counted in the total)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quick-release clamp, Arca-Swiss (DAZ's cheaper 'option 2')</t>
+    <t xml:space="preserve">4. OPTIONAL UPGRADE – wheel buttons &amp; magnetic paddles (NOT counted in the total)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wireless button board (2.4 GHz zero-delay arcade encoder)</t>
   </si>
   <si>
     <t xml:space="preserve">Removed – optional</t>
   </si>
   <si>
-    <t xml:space="preserve">Only lets you slide the whole wheelbase off the desk without tools – DAZ himself says the one he used is pricey (his first pick, a FANAUE lever clamp, is ≈ AUD 40+). Without it, fix the base straight to your desk mount; check DAZ's guide for which screw holds the plate.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cheap Arca-Swiss clamps US$5–11 (2026).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quick-release plate, Arca-Swiss, 100 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Goes with the clamp above.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wireless button board (2.4 GHz zero-delay arcade encoder)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only needed for buttons and paddles on the wheel. The H-shifter (with its sequential mode) already handles gear changes, and things like pit limiter or wipers can go on the keyboard. Part of the wheel-buttons upgrade (≈ AUD 35 for everything from the wireless board down).</t>
+    <t xml:space="preserve">Only needed for buttons and paddles on the wheel. The H-shifter (with its sequential mode) already handles gear changes, and things like pit limiter or wipers can go on the keyboard. Part of the wheel-buttons upgrade (≈ AUD 35 for this whole section).</t>
   </si>
   <si>
     <t xml:space="preserve">A listing with this exact title showed US$4.29 sale / US$17.58 full price in a 2026 search. Estimate AUD 15.</t>
@@ -364,7 +364,7 @@
     <t xml:space="preserve">2 sets</t>
   </si>
   <si>
-    <t xml:space="preserve">Part of the wheel-buttons upgrade (≈ AUD 35 for everything from the wireless board down).</t>
+    <t xml:space="preserve">Part of the wheel-buttons upgrade (≈ AUD 35 for this whole section).</t>
   </si>
   <si>
     <t xml:space="preserve">DAZ's link: US$1.91 per set (May 2025) ≈ AUD 3.</t>
@@ -382,7 +382,7 @@
     <t xml:space="preserve">AA battery holder, 2 × AA</t>
   </si>
   <si>
-    <t xml:space="preserve">Powers the wireless board. Part of the wheel-buttons upgrade (≈ AUD 35 for everything from the wireless board down).</t>
+    <t xml:space="preserve">Powers the wireless board. Part of the wheel-buttons upgrade (≈ AUD 35 for this whole section).</t>
   </si>
   <si>
     <t xml:space="preserve">Typical listing US$0.50–1.</t>
@@ -391,7 +391,7 @@
     <t xml:space="preserve">Limit switches with roller lever (paddles), 10-pack</t>
   </si>
   <si>
-    <t xml:space="preserve">Paddle switches. DAZ's shifter uses a 10-pack of roller-lever switches and leaves 5 spare – if they're the same size (compare the photos), this costs nothing extra. Part of the wheel-buttons upgrade (≈ AUD 35 for everything from the wireless board down).</t>
+    <t xml:space="preserve">Paddle switches. DAZ's shifter uses a 10-pack of roller-lever switches and leaves 5 spare – if they're the same size (compare the photos), this costs nothing extra. Part of the wheel-buttons upgrade (≈ AUD 35 for this whole section).</t>
   </si>
   <si>
     <t xml:space="preserve">DAZ's link: US$3.57 per 10 (May 2025) ≈ AUD 5.70.</t>
@@ -406,16 +406,16 @@
     <t xml:space="preserve">Supermarket / Kmart</t>
   </si>
   <si>
-    <t xml:space="preserve">For the wireless board. Part of the wheel-buttons upgrade (≈ AUD 35 for everything from the wireless board down).</t>
+    <t xml:space="preserve">For the wireless board. Part of the wheel-buttons upgrade (≈ AUD 35 for this whole section).</t>
   </si>
   <si>
     <t xml:space="preserve">Supermarket price.</t>
   </si>
   <si>
-    <t xml:space="preserve">Add-ons subtotal (not counted)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total if you add all of section 4 back</t>
+    <t xml:space="preserve">Upgrade subtotal (not counted)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total with the buttons upgrade</t>
   </si>
   <si>
     <t xml:space="preserve">5. NOT COUNTED – things you may already have</t>
@@ -478,10 +478,13 @@
     <t xml:space="preserve">• Reuse an old 19–20 V laptop charger (ideally 120 W+) instead of buying the 24 V PSU: −AUD 20 (lower maximum force).</t>
   </si>
   <si>
-    <t xml:space="preserve">• Get a broken hoverboard for free (friends, Buy Nothing groups, council clean-ups): −AUD 30.</t>
+    <t xml:space="preserve">• Skip the quick release and bolt the base straight to your desk mount: −AUD 23 (only if DAZ's guide shows a solid way to do it).</t>
   </si>
   <si>
     <t xml:space="preserve">• Building the shifter and pedals too? Buy the screws once – several sizes repeat: −AUD 5 or more.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Adding the buttons later? Use 2 of the 5 spare roller-lever switches from the shifter's 10-pack for the paddles (if they're the same size): the upgrade drops to ≈ AUD 29.50.</t>
   </si>
   <si>
     <t xml:space="preserve">• Order the controller, rim and encoder in AliExpress's 11.11 sale (11 November).</t>
@@ -783,6 +786,10 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -809,10 +816,6 @@
     </xf>
     <xf numFmtId="164" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -1109,7 +1112,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -1144,12 +1147,12 @@
         <v>3</v>
       </c>
       <c r="E3" s="6" t="n">
-        <f aca="false">E39</f>
-        <v>196</v>
+        <f aca="false">E41</f>
+        <v>189</v>
       </c>
       <c r="F3" s="3" t="str">
         <f aca="false">IF(E3&lt;=B3,"UNDER BUDGET – $"&amp;TEXT(B3-E3,"0.00")&amp;" spare","OVER BUDGET by $"&amp;TEXT(E3-B3,"0.00"))</f>
-        <v>UNDER BUDGET – $4.00 spare</v>
+        <v>UNDER BUDGET – $11.00 spare</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1231,42 +1234,40 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="66.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C8" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E8" s="12" t="n">
         <f aca="false">C8*D8</f>
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F8" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="H8" s="16"/>
+      <c r="I8" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="J8" s="9" t="s">
         <v>26</v>
-      </c>
-      <c r="I8" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="J8" s="9" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>16</v>
@@ -1282,7 +1283,7 @@
         <v>20</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G9" s="9" t="s">
         <v>18</v>
@@ -1291,15 +1292,15 @@
         <v>19</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>16</v>
@@ -1315,7 +1316,7 @@
         <v>38</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G10" s="9" t="s">
         <v>18</v>
@@ -1324,15 +1325,15 @@
         <v>19</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>16</v>
@@ -1348,7 +1349,7 @@
         <v>2</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G11" s="9" t="s">
         <v>18</v>
@@ -1357,15 +1358,15 @@
         <v>19</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="J11" s="9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>16</v>
@@ -1381,7 +1382,7 @@
         <v>2.5</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G12" s="9" t="s">
         <v>18</v>
@@ -1390,15 +1391,15 @@
         <v>19</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B13" s="9" t="s">
         <v>16</v>
@@ -1414,7 +1415,7 @@
         <v>3.5</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G13" s="9" t="s">
         <v>18</v>
@@ -1423,15 +1424,15 @@
         <v>19</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="66.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>16</v>
@@ -1447,7 +1448,7 @@
         <v>20</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G14" s="9" t="s">
         <v>18</v>
@@ -1456,18 +1457,18 @@
         <v>19</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C15" s="10" t="n">
         <v>1</v>
@@ -1480,7 +1481,7 @@
         <v>2.5</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G15" s="9" t="s">
         <v>18</v>
@@ -1489,15 +1490,15 @@
         <v>19</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B16" s="9" t="s">
         <v>16</v>
@@ -1513,7 +1514,7 @@
         <v>6</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G16" s="9" t="s">
         <v>18</v>
@@ -1522,18 +1523,18 @@
         <v>19</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J16" s="9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C17" s="10" t="n">
         <v>1</v>
@@ -1546,7 +1547,7 @@
         <v>4.5</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G17" s="9" t="s">
         <v>18</v>
@@ -1555,126 +1556,128 @@
         <v>19</v>
       </c>
       <c r="I17" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="J17" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="66.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="J17" s="9" t="s">
+      <c r="B18" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <f aca="false">C18*D18</f>
+        <v>16</v>
+      </c>
+      <c r="F18" s="13" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="16" t="s">
+      <c r="G18" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I18" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="18" t="n">
-        <f aca="false">SUM(E7:E17)</f>
-        <v>179</v>
-      </c>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
+      <c r="J18" s="9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E19" s="12" t="n">
+        <f aca="false">C19*D19</f>
+        <v>7</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H19" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I19" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="J19" s="9" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-    </row>
-    <row r="21" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="C21" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="12" t="n">
-        <f aca="false">C21*D21</f>
-        <v>1</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="G21" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="H21" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I21" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="J21" s="9" t="s">
+      <c r="A20" s="17" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9" t="s">
+      <c r="B20" s="18"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="19" t="n">
+        <f aca="false">SUM(E7:E19)</f>
+        <v>172</v>
+      </c>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="18"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
+    </row>
+    <row r="23" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C22" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="12" t="n">
-        <f aca="false">C22*D22</f>
-        <v>1</v>
-      </c>
-      <c r="F22" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="G22" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="H22" s="14" t="s">
+      <c r="B23" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>16</v>
-      </c>
       <c r="C23" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D23" s="11" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E23" s="12" t="n">
         <f aca="false">C23*D23</f>
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G23" s="9" t="s">
         <v>18</v>
@@ -1682,48 +1685,50 @@
       <c r="H23" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="I23" s="9"/>
+      <c r="I23" s="9" t="s">
+        <v>73</v>
+      </c>
       <c r="J23" s="9" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C24" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="11" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E24" s="12" t="n">
         <f aca="false">C24*D24</f>
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G24" s="9" t="s">
         <v>18</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>19</v>
+        <v>77</v>
       </c>
       <c r="I24" s="9"/>
       <c r="J24" s="9" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="C25" s="10" t="n">
         <v>1</v>
@@ -1736,7 +1741,7 @@
         <v>1.5</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G25" s="9" t="s">
         <v>18</v>
@@ -1746,28 +1751,28 @@
       </c>
       <c r="I25" s="9"/>
       <c r="J25" s="9" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="B26" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B26" s="9" t="s">
-        <v>77</v>
-      </c>
       <c r="C26" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="11" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E26" s="12" t="n">
         <f aca="false">C26*D26</f>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G26" s="9" t="s">
         <v>18</v>
@@ -1777,28 +1782,28 @@
       </c>
       <c r="I26" s="9"/>
       <c r="J26" s="9" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C27" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="11" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E27" s="12" t="n">
         <f aca="false">C27*D27</f>
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G27" s="9" t="s">
         <v>18</v>
@@ -1808,15 +1813,15 @@
       </c>
       <c r="I27" s="9"/>
       <c r="J27" s="9" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C28" s="10" t="n">
         <v>1</v>
@@ -1829,7 +1834,7 @@
         <v>1</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G28" s="9" t="s">
         <v>18</v>
@@ -1839,15 +1844,15 @@
       </c>
       <c r="I28" s="9"/>
       <c r="J28" s="9" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C29" s="10" t="n">
         <v>1</v>
@@ -1860,7 +1865,7 @@
         <v>1</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G29" s="9" t="s">
         <v>18</v>
@@ -1870,28 +1875,28 @@
       </c>
       <c r="I29" s="9"/>
       <c r="J29" s="9" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="C30" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D30" s="11" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E30" s="12" t="n">
         <f aca="false">C30*D30</f>
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G30" s="9" t="s">
         <v>18</v>
@@ -1901,28 +1906,28 @@
       </c>
       <c r="I30" s="9"/>
       <c r="J30" s="9" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>16</v>
+        <v>82</v>
       </c>
       <c r="C31" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E31" s="12" t="n">
         <f aca="false">C31*D31</f>
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G31" s="9" t="s">
         <v>18</v>
@@ -1932,223 +1937,219 @@
       </c>
       <c r="I31" s="9"/>
       <c r="J31" s="9" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="C32" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D32" s="11" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="E32" s="12" t="n">
         <f aca="false">C32*D32</f>
+        <v>1.5</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H32" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I32" s="9"/>
+      <c r="J32" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C33" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="11" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E33" s="12" t="n">
+        <f aca="false">C33*D33</f>
+        <v>1.5</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H33" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C34" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="11" t="n">
         <v>2.5</v>
       </c>
-      <c r="F32" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="G32" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="H32" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="I32" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="J32" s="9" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="B33" s="17"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="18" t="n">
-        <f aca="false">SUM(E21:E32)</f>
+      <c r="E34" s="12" t="n">
+        <f aca="false">C34*D34</f>
+        <v>2.5</v>
+      </c>
+      <c r="F34" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="H34" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="I34" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="J34" s="9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="B35" s="18"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="19" t="n">
+        <f aca="false">SUM(E23:E34)</f>
         <v>16</v>
       </c>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="17"/>
-      <c r="I33" s="17"/>
-      <c r="J33" s="17"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="B35" s="8"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
-      <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="8"/>
-      <c r="I35" s="8"/>
-      <c r="J35" s="8"/>
-    </row>
-    <row r="36" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="B36" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="C36" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" s="12" t="n">
-        <f aca="false">C36*D36</f>
-        <v>1</v>
-      </c>
-      <c r="F36" s="19" t="s">
-        <v>94</v>
-      </c>
-      <c r="G36" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="H36" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="I36" s="9" t="s">
+      <c r="F35" s="18"/>
+      <c r="G35" s="18"/>
+      <c r="H35" s="18"/>
+      <c r="I35" s="18"/>
+      <c r="J35" s="18"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="J36" s="9" t="s">
+      <c r="B37" s="8"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="8"/>
+      <c r="I37" s="8"/>
+      <c r="J37" s="8"/>
+    </row>
+    <row r="38" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="9" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="16" t="s">
+      <c r="B38" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C38" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="12" t="n">
+        <f aca="false">C38*D38</f>
+        <v>1</v>
+      </c>
+      <c r="F38" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="17"/>
-      <c r="E37" s="18" t="n">
-        <f aca="false">SUM(E36:E36)</f>
-        <v>1</v>
-      </c>
-      <c r="F37" s="17"/>
-      <c r="G37" s="17"/>
-      <c r="H37" s="17"/>
-      <c r="I37" s="17"/>
-      <c r="J37" s="17"/>
-    </row>
-    <row r="39" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="20" t="s">
+      <c r="G38" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="B39" s="20"/>
-      <c r="C39" s="20"/>
-      <c r="D39" s="20"/>
-      <c r="E39" s="21" t="n">
-        <f aca="false">E18+E33+E37</f>
-        <v>196</v>
-      </c>
-      <c r="F39" s="20"/>
-      <c r="G39" s="20"/>
-      <c r="H39" s="20"/>
-      <c r="I39" s="20"/>
-      <c r="J39" s="20"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="8" t="s">
+      <c r="H38" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="B41" s="8"/>
-      <c r="C41" s="8"/>
-      <c r="D41" s="8"/>
-      <c r="E41" s="8"/>
-      <c r="F41" s="8"/>
-      <c r="G41" s="8"/>
-      <c r="H41" s="8"/>
-      <c r="I41" s="8"/>
-      <c r="J41" s="8"/>
-    </row>
-    <row r="42" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="9" t="s">
+      <c r="I38" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="B42" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="C42" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" s="11" t="n">
-        <v>16</v>
-      </c>
-      <c r="E42" s="12" t="n">
-        <f aca="false">C42*D42</f>
-        <v>16</v>
-      </c>
-      <c r="F42" s="22" t="s">
+      <c r="J38" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="G42" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="H42" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I42" s="9" t="s">
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="J42" s="9" t="s">
+      <c r="B39" s="18"/>
+      <c r="C39" s="18"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="19" t="n">
+        <f aca="false">SUM(E38:E38)</f>
+        <v>1</v>
+      </c>
+      <c r="F39" s="18"/>
+      <c r="G39" s="18"/>
+      <c r="H39" s="18"/>
+      <c r="I39" s="18"/>
+      <c r="J39" s="18"/>
+    </row>
+    <row r="41" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="21" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="9" t="s">
+      <c r="B41" s="21"/>
+      <c r="C41" s="21"/>
+      <c r="D41" s="21"/>
+      <c r="E41" s="22" t="n">
+        <f aca="false">E20+E35+E39</f>
+        <v>189</v>
+      </c>
+      <c r="F41" s="21"/>
+      <c r="G41" s="21"/>
+      <c r="H41" s="21"/>
+      <c r="I41" s="21"/>
+      <c r="J41" s="21"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="B43" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="C43" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="E43" s="12" t="n">
-        <f aca="false">C43*D43</f>
-        <v>7</v>
-      </c>
-      <c r="F43" s="22" t="s">
-        <v>103</v>
-      </c>
-      <c r="G43" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="H43" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I43" s="9" t="s">
+      <c r="B43" s="8"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="8"/>
+      <c r="F43" s="8"/>
+      <c r="G43" s="8"/>
+      <c r="H43" s="8"/>
+      <c r="I43" s="8"/>
+      <c r="J43" s="8"/>
+    </row>
+    <row r="44" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="9" t="s">
         <v>107</v>
-      </c>
-      <c r="J43" s="9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="9" t="s">
-        <v>108</v>
       </c>
       <c r="B44" s="9" t="s">
         <v>16</v>
@@ -2163,8 +2164,8 @@
         <f aca="false">C44*D44</f>
         <v>15</v>
       </c>
-      <c r="F44" s="22" t="s">
-        <v>103</v>
+      <c r="F44" s="23" t="s">
+        <v>108</v>
       </c>
       <c r="G44" s="9" t="s">
         <v>18</v>
@@ -2179,7 +2180,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="9" t="s">
         <v>111</v>
       </c>
@@ -2196,8 +2197,8 @@
         <f aca="false">C45*D45</f>
         <v>6</v>
       </c>
-      <c r="F45" s="22" t="s">
-        <v>103</v>
+      <c r="F45" s="23" t="s">
+        <v>108</v>
       </c>
       <c r="G45" s="9" t="s">
         <v>18</v>
@@ -2212,7 +2213,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="9" t="s">
         <v>115</v>
       </c>
@@ -2229,8 +2230,8 @@
         <f aca="false">C46*D46</f>
         <v>5</v>
       </c>
-      <c r="F46" s="22" t="s">
-        <v>103</v>
+      <c r="F46" s="23" t="s">
+        <v>108</v>
       </c>
       <c r="G46" s="9" t="s">
         <v>18</v>
@@ -2262,8 +2263,8 @@
         <f aca="false">C47*D47</f>
         <v>1.5</v>
       </c>
-      <c r="F47" s="22" t="s">
-        <v>103</v>
+      <c r="F47" s="23" t="s">
+        <v>108</v>
       </c>
       <c r="G47" s="9" t="s">
         <v>18</v>
@@ -2283,7 +2284,7 @@
         <v>121</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C48" s="10" t="n">
         <v>1</v>
@@ -2295,8 +2296,8 @@
         <f aca="false">C48*D48</f>
         <v>5.5</v>
       </c>
-      <c r="F48" s="22" t="s">
-        <v>103</v>
+      <c r="F48" s="23" t="s">
+        <v>108</v>
       </c>
       <c r="G48" s="9" t="s">
         <v>18</v>
@@ -2316,7 +2317,7 @@
         <v>124</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C49" s="10" t="n">
         <v>1</v>
@@ -2328,13 +2329,13 @@
         <f aca="false">C49*D49</f>
         <v>2</v>
       </c>
-      <c r="F49" s="22" t="s">
+      <c r="F49" s="23" t="s">
         <v>125</v>
       </c>
       <c r="G49" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="H49" s="23"/>
+      <c r="H49" s="16"/>
       <c r="I49" s="9" t="s">
         <v>127</v>
       </c>
@@ -2343,29 +2344,29 @@
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="16" t="s">
+      <c r="A50" s="17" t="s">
         <v>129</v>
       </c>
-      <c r="B50" s="17"/>
-      <c r="C50" s="17"/>
-      <c r="D50" s="17"/>
-      <c r="E50" s="18" t="n">
-        <f aca="false">SUM(E42:E49)</f>
-        <v>58</v>
-      </c>
-      <c r="F50" s="17"/>
-      <c r="G50" s="17"/>
-      <c r="H50" s="17"/>
-      <c r="I50" s="17"/>
-      <c r="J50" s="17"/>
+      <c r="B50" s="18"/>
+      <c r="C50" s="18"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="19" t="n">
+        <f aca="false">SUM(E44:E49)</f>
+        <v>35</v>
+      </c>
+      <c r="F50" s="18"/>
+      <c r="G50" s="18"/>
+      <c r="H50" s="18"/>
+      <c r="I50" s="18"/>
+      <c r="J50" s="18"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
         <v>130</v>
       </c>
       <c r="E51" s="6" t="n">
-        <f aca="false">E39+E50</f>
-        <v>254</v>
+        <f aca="false">E41+E50</f>
+        <v>224</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2405,7 +2406,7 @@
       <c r="G54" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="H54" s="23"/>
+      <c r="H54" s="16"/>
       <c r="I54" s="9" t="s">
         <v>136</v>
       </c>
@@ -2436,7 +2437,7 @@
       <c r="G55" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="H55" s="23"/>
+      <c r="H55" s="16"/>
       <c r="I55" s="9" t="s">
         <v>141</v>
       </c>
@@ -2467,7 +2468,7 @@
       <c r="G56" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="H56" s="23"/>
+      <c r="H56" s="16"/>
       <c r="I56" s="9" t="s">
         <v>145</v>
       </c>
@@ -2476,29 +2477,29 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="16" t="s">
+      <c r="A57" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="B57" s="17"/>
-      <c r="C57" s="17"/>
-      <c r="D57" s="17"/>
-      <c r="E57" s="18" t="n">
+      <c r="B57" s="18"/>
+      <c r="C57" s="18"/>
+      <c r="D57" s="18"/>
+      <c r="E57" s="19" t="n">
         <f aca="false">SUM(E54:E56)</f>
         <v>30</v>
       </c>
-      <c r="F57" s="17"/>
-      <c r="G57" s="17"/>
-      <c r="H57" s="17"/>
-      <c r="I57" s="17"/>
-      <c r="J57" s="17"/>
+      <c r="F57" s="18"/>
+      <c r="G57" s="18"/>
+      <c r="H57" s="18"/>
+      <c r="I57" s="18"/>
+      <c r="J57" s="18"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
         <v>148</v>
       </c>
       <c r="E58" s="6" t="n">
-        <f aca="false">E39+E57</f>
-        <v>226</v>
+        <f aca="false">E41+E57</f>
+        <v>219</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2571,33 +2572,33 @@
       <c r="I64" s="25"/>
       <c r="J64" s="25"/>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="8" t="s">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="25" t="s">
         <v>154</v>
       </c>
-      <c r="B66" s="8"/>
-      <c r="C66" s="8"/>
-      <c r="D66" s="8"/>
-      <c r="E66" s="8"/>
-      <c r="F66" s="8"/>
-      <c r="G66" s="8"/>
-      <c r="H66" s="8"/>
-      <c r="I66" s="8"/>
-      <c r="J66" s="8"/>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="26" t="s">
+      <c r="B65" s="25"/>
+      <c r="C65" s="25"/>
+      <c r="D65" s="25"/>
+      <c r="E65" s="25"/>
+      <c r="F65" s="25"/>
+      <c r="G65" s="25"/>
+      <c r="H65" s="25"/>
+      <c r="I65" s="25"/>
+      <c r="J65" s="25"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="B67" s="26"/>
-      <c r="C67" s="26"/>
-      <c r="D67" s="26"/>
-      <c r="E67" s="26"/>
-      <c r="F67" s="26"/>
-      <c r="G67" s="26"/>
-      <c r="H67" s="26"/>
-      <c r="I67" s="26"/>
-      <c r="J67" s="26"/>
+      <c r="B67" s="8"/>
+      <c r="C67" s="8"/>
+      <c r="D67" s="8"/>
+      <c r="E67" s="8"/>
+      <c r="F67" s="8"/>
+      <c r="G67" s="8"/>
+      <c r="H67" s="8"/>
+      <c r="I67" s="8"/>
+      <c r="J67" s="8"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="26" t="s">
@@ -2669,18 +2670,33 @@
       <c r="I72" s="26"/>
       <c r="J72" s="26"/>
     </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="26" t="s">
+        <v>161</v>
+      </c>
+      <c r="B73" s="26"/>
+      <c r="C73" s="26"/>
+      <c r="D73" s="26"/>
+      <c r="E73" s="26"/>
+      <c r="F73" s="26"/>
+      <c r="G73" s="26"/>
+      <c r="H73" s="26"/>
+      <c r="I73" s="26"/>
+      <c r="J73" s="26"/>
+    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A61:J61"/>
     <mergeCell ref="A62:J62"/>
     <mergeCell ref="A63:J63"/>
     <mergeCell ref="A64:J64"/>
-    <mergeCell ref="A67:J67"/>
+    <mergeCell ref="A65:J65"/>
     <mergeCell ref="A68:J68"/>
     <mergeCell ref="A69:J69"/>
     <mergeCell ref="A70:J70"/>
     <mergeCell ref="A71:J71"/>
     <mergeCell ref="A72:J72"/>
+    <mergeCell ref="A73:J73"/>
   </mergeCells>
   <conditionalFormatting sqref="F3">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -2692,36 +2708,35 @@
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="H7" r:id="rId1" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H8" r:id="rId2" display="Gumtree search: hoverboard"/>
-    <hyperlink ref="H9" r:id="rId3" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H10" r:id="rId4" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H11" r:id="rId5" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H12" r:id="rId6" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H13" r:id="rId7" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H14" r:id="rId8" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H15" r:id="rId9" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H16" r:id="rId10" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H17" r:id="rId11" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H21" r:id="rId12" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H22" r:id="rId13" display="AliExpress search: M5 washer"/>
-    <hyperlink ref="H23" r:id="rId14" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H24" r:id="rId15" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H25" r:id="rId16" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H26" r:id="rId17" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H27" r:id="rId18" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H28" r:id="rId19" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H29" r:id="rId20" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H30" r:id="rId21" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H31" r:id="rId22" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H32" r:id="rId23" display="Bunnings search: 3 mm nails"/>
-    <hyperlink ref="H36" r:id="rId24" display="AliExpress search: 2.2k resistor"/>
-    <hyperlink ref="H42" r:id="rId25" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H43" r:id="rId26" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H44" r:id="rId27" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H45" r:id="rId28" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H46" r:id="rId29" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H47" r:id="rId30" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H48" r:id="rId31" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H9" r:id="rId2" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H10" r:id="rId3" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H11" r:id="rId4" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H12" r:id="rId5" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H13" r:id="rId6" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H14" r:id="rId7" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H15" r:id="rId8" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H16" r:id="rId9" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H17" r:id="rId10" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H18" r:id="rId11" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H19" r:id="rId12" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H23" r:id="rId13" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H24" r:id="rId14" display="AliExpress search: M5 washer"/>
+    <hyperlink ref="H25" r:id="rId15" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H26" r:id="rId16" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H27" r:id="rId17" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H28" r:id="rId18" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H29" r:id="rId19" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H30" r:id="rId20" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H31" r:id="rId21" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H32" r:id="rId22" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H33" r:id="rId23" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H34" r:id="rId24" display="Bunnings search: 3 mm nails"/>
+    <hyperlink ref="H38" r:id="rId25" display="AliExpress search: 2.2k resistor"/>
+    <hyperlink ref="H44" r:id="rId26" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H45" r:id="rId27" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H46" r:id="rId28" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H47" r:id="rId29" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H48" r:id="rId30" display="AliExpress – DAZ's link"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Add combined best-value list, backup links and listing checks
- New combined list for all three builds: shared screws bought once, free
  parts scrounged, optional buttons upgrade, and a section of cheaper
  trade-offs. About AUD 326, or AUD 194 with every trade-off.
- Every part now has a main link and a backup link. Generic parts link to
  an any-seller AliExpress search; parts DAZ's prints depend on keep his
  listing.
- New "Listing check" column records whether each DAZ link still leads to
  a live product page.
- Per-build lists: skateboard bearings, bike cables and the pedal base
  moved to "free if you can scrounge them". Shifter about AUD 66, pedals
  about AUD 86, wheel unchanged at AUD 189.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QEYLvGWigrKvVwvVek2yBU
</commit_message>
<xml_diff>
--- a/parts-lists/DAZ_racing_V2_steering_wheel_budget_parts_list_AUD.xlsx
+++ b/parts-lists/DAZ_racing_V2_steering_wheel_budget_parts_list_AUD.xlsx
@@ -8,10 +8,10 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Budget parts list" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Parts list" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Budget parts list'!$5:$5</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Parts list'!$5:$5</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,12 +23,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="195">
   <si>
     <t xml:space="preserve">DAZ Racing V2 Steering Wheel – budget parts list (AUD)</t>
   </si>
   <si>
-    <t xml:space="preserve">Budget version of DAZ's parts list, re-priced for Australia. Prices are estimates in AUD incl. 10% GST, checked 2 Oct 2026 – AliExpress prices change daily, so edit the blue cells and everything re-totals.</t>
+    <t xml:space="preserve">Prices are estimates in AUD incl. 10% GST, checked 3 Oct 2026. AliExpress prices change daily – edit the blue cells and everything re-totals. Every part has a main link and a backup link in case a listing sells out.</t>
   </si>
   <si>
     <t xml:space="preserve">Budget (AUD) – edit the yellow cell</t>
@@ -58,7 +58,13 @@
     <t xml:space="preserve">Where to buy</t>
   </si>
   <si>
-    <t xml:space="preserve">Link</t>
+    <t xml:space="preserve">Main link</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backup link</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listing check</t>
   </si>
   <si>
     <t xml:space="preserve">Notes</t>
@@ -76,7 +82,7 @@
     <t xml:space="preserve">1</t>
   </si>
   <si>
-    <t xml:space="preserve">Kept – cheapest board that runs FFBeast</t>
+    <t xml:space="preserve">Kept – DAZ's exact part</t>
   </si>
   <si>
     <t xml:space="preserve">AliExpress</t>
@@ -85,10 +91,16 @@
     <t xml:space="preserve">AliExpress – DAZ's link</t>
   </si>
   <si>
-    <t xml:space="preserve">Runs the FFBeast firmware for free in its 'light' mode – the paid licence only adds extra settings and buttons wired straight to the controller, which DAZ's design doesn't use. Check the listing includes the brake resistor. DAZ's 'America' link is an ODESC V4.2 (also FFBeast-compatible); only take it if it's clearly cheaper, since the XDrive Mini is what his list is built around.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DAZ's link: €29.92 sale (May 2025) ≈ AUD 44 incl. GST. 2026 US-store listings US$37–41 ≈ AUD 59–65 incl. GST. Estimate AUD 50 (between the two – check the live price).</t>
+    <t xml:space="preserve">AliExpress search: MKS XDrive Mini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Live (3 Oct 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The one part with no cheap substitute. Runs FFBeast's free 'light' mode – the paid licence only adds extras DAZ's design doesn't use. Check the listing includes the brake resistor. Cheapest time to buy: AliExpress's 11.11 sale (11 Nov) or with new-user coupons.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DAZ's link: €29.92 sale (May 2025) ≈ AUD 44 incl. GST. 2026 US-store listings US$37–41 ≈ AUD 59–65 incl. GST. Estimate AUD 50.</t>
   </si>
   <si>
     <t xml:space="preserve">6.5" hoverboard motor</t>
@@ -100,19 +112,22 @@
     <t xml:space="preserve">You already own it</t>
   </si>
   <si>
-    <t xml:space="preserve">Before you print, check it's a 6.5" (165 mm) motor that spins freely and doesn't grind – DAZ's mount is sized for 6.5" motors.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">You already have it, so it costs nothing.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rotary encoder E6B2-CWZ6C (6 mm shaft, NPN output)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kept – cheapest variant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Any resolution from 600 P/R up works (FFBeast asks for ≥1000 counts per turn, and 600 P/R already gives 2,400). DAZ used 2000 P/R – take it if it's only a dollar or two more. NPN output, so it needs the pull-up resistors in section 3.</t>
+    <t xml:space="preserve">Check it's a 6.5" (165 mm) motor that spins freely without grinding – DAZ's mount is sized for 6.5".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You own it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rotary encoder E6B2-CWZ6C, 1000–2000 P/R (6 mm shaft, NPN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: E6B2-CWZ6C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Link OK – page not auto-checked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DAZ's encoder mount is made for this body, and high resolution gives smooth force feedback, so it stays. 1000 P/R is plenty if it's cheaper (FFBeast asks for ≥1000 counts per turn). NPN output – needs the pull-up resistors below.</t>
   </si>
   <si>
     <t xml:space="preserve">DAZ's link: US$13.53 (May 2025) ≈ AUD 21.50 incl. GST; similar 2026 listings US$13.70–15.30.</t>
@@ -121,22 +136,31 @@
     <t xml:space="preserve">Steering wheel rim, 13" / 330 mm flat, aluminium + PVC</t>
   </si>
   <si>
-    <t xml:space="preserve">Kept – PVC version</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DAZ: "get this, I can't guarantee this build works with a different one" – so keep his wheel, but pick the PVC (not suede) option, which is the cheapest.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 AliExpress: 13" PVC flat wheels US$20–27 ≈ AUD 32–43 incl. GST (suede ones US$47–55). Estimate AUD 38.</t>
+    <t xml:space="preserve">Kept – DAZ's exact part (PVC version)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: 13" flat wheel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DAZ: "get this, I can't guarantee this build works with a different one". Pick the PVC option – it's the cheapest. If his listing ever disappears, choose a 13-inch flat-dish wheel with the 6 × 70 mm bolt pattern.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 AliExpress: 13" PVC flat wheels US$20–27 ≈ AUD 32–43 incl. GST (suede US$47–55). Estimate AUD 38.</t>
   </si>
   <si>
     <t xml:space="preserve">GT2 timing pulley, 20T, 6 mm bore, 6 mm belt</t>
   </si>
   <si>
-    <t xml:space="preserve">Kept</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Goes on the encoder shaft.</t>
+    <t xml:space="preserve">Cheaper – any seller, same size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: GT2 20T 6 mm bore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Search – in-stock sellers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standard part – any seller with these sizes. Goes on the encoder shaft.</t>
   </si>
   <si>
     <t xml:space="preserve">Typical listing US$1–1.50.</t>
@@ -145,13 +169,19 @@
     <t xml:space="preserve">GT2 closed-loop belt, 212 mm, 6 mm wide</t>
   </si>
   <si>
-    <t xml:space="preserve">Drives the encoder from the motor.</t>
+    <t xml:space="preserve">AliExpress search: GT2 belt 212 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Must be a closed loop, 212 mm long, 6 mm wide.</t>
   </si>
   <si>
     <t xml:space="preserve">Typical listing US$1–2.</t>
   </si>
   <si>
-    <t xml:space="preserve">GT2 idler, 20T, 5 mm bore, 6 mm wide</t>
+    <t xml:space="preserve">GT2 idler, 20T toothed, 5 mm bore, 6 mm wide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: GT2 idler 20T 5 mm</t>
   </si>
   <si>
     <t xml:space="preserve">Keeps the encoder belt tight.</t>
@@ -160,16 +190,16 @@
     <t xml:space="preserve">DAZ's link: US$2.24 (May 2025) ≈ AUD 3.55 incl. GST.</t>
   </si>
   <si>
-    <t xml:space="preserve">Power supply, 24 V 10 A (240 W)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kept – cheapest listing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Choose the 24V 10A option with an AU plug. Already own an old laptop charger (19–20 V, ideally 120 W or more)? FFBeast says supplies from 12 V up work at lighter force settings – use it and this line is $0. If the PSU arrives as a bare metal box with screw terminals, the 240 V side must be wired and covered properly; not confident? Buy the enclosed 'adapter' version.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DAZ's link: US$11.15 (May 2025) ≈ AUD 18 incl. GST. Estimate AUD 20 for the 24V 10A option.</t>
+    <t xml:space="preserve">Power supply, 24 V 10 A (240 W), AU plug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: 24V 10A power supply</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The full 240 W gives the full force. Pick an enclosed 'adapter' type with an AU plug, so there's no 240 V wiring to do. Any brand works.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DAZ's link: US$11.15 (May 2025) ≈ AUD 18 incl. GST. Estimate AUD 20.</t>
   </si>
   <si>
     <t xml:space="preserve">XT60 connector pair (male + female)</t>
@@ -178,136 +208,187 @@
     <t xml:space="preserve">1 pair</t>
   </si>
   <si>
+    <t xml:space="preserve">Cheaper – any seller, same size (smallest pack)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: XT60 pair</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power plug between the PSU and the controller – one pair is enough.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small packs ≈ US$1–2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor axle clamp, 16 × 16 mm cross clamp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: 16 mm cross clamp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part of DAZ's V2 mount – his printed parts are designed around it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typical listing US$3–5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aluminium tube, 16 mm OD (cut to 100 mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kept – DAZ's exact part (shortest length)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: 16 mm aluminium tube</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pick 16 mm outside diameter and the shortest length (e.g. 250 mm); cut to 100 mm with a hacksaw.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typical 250 mm length US$2–3.50.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quick-release clamp, Arca-Swiss (DAZ's cheaper 'option 2')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kept – DAZ's exact part (cheaper option)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: Arca-Swiss clamp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How DAZ's V2 base attaches to the desk or your frame ("aluminum Quick-Release to detach from the desk"). His listing is titled as a plate – pick the clamp option; any Arca-Swiss clamp grips the plate below.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cheap Arca-Swiss clamps US$5–11 (2026) ≈ AUD 8–17.50 incl. GST.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quick-release plate, Arca-Swiss, 100 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: Arca plate 100 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Goes with the clamp above.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal – parts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. NUTS &amp; BOLTS (DAZ's list)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M5 nuts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cheaper – any seller, same size (small pack)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: M5 nut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pick the exact size and the smallest quantity. Plain steel is cheaper than stainless and fine indoors. Bunnings has most sizes today but costs 2–3× more.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small AliExpress pack ≈ AUD 1–2.50.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M5 washers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: M5 washer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M5 × 20 cap screw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: M5x20 socket head</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M5 × 25 socket head screws</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: M5x25 socket head</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M5 × 40 socket head screws</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: M5x40 socket head</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3 × 10 socket head screws</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: M3x10 socket head</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3 × 12 self-tapping screws</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: M3x12 self-tapping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2.5 × 6 self-tapping screws</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: M2.5x6 self-tapping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6 nuts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: M6 nut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6 × 30 countersunk screws</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: M6x30 countersunk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M6 × 45 countersunk screw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: M6x45 countersunk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 mm nails</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kept – smallest pack</t>
   </si>
   <si>
-    <t xml:space="preserve">Power plug between the PSU and the controller. One pair is enough, so buy the smallest pack.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Small packs ≈ US$1–2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Motor axle clamp, 16 × 16 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DAZ lists it for the upgraded V2 mount / quick release. It's cheap and the V2 printed parts are designed around it, so it stays.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typical listing US$3–5.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aluminium tube, 16 mm OD (cut to 100 mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kept – shortest length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buy the shortest length offered (e.g. 250 mm) and cut it to 100 mm with a hacksaw.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typical 250 mm length US$2–3.50.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quick-release clamp, Arca-Swiss (DAZ's cheaper 'option 2')</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kept – DAZ's cheaper option</t>
-  </si>
-  <si>
-    <t xml:space="preserve">This is how DAZ's V2 base attaches to the desk (his "aluminum Quick-Release to detach from the desk"), so it's back in now that the motor costs nothing – the build goes together as designed. His first pick, a FANAUE lever clamp, is ≈ AUD 40+. This cheaper listing is titled as a plate: pick its clamp option if it has one; any Arca-Swiss clamp grips the 100 mm plate below.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cheap Arca-Swiss clamps US$5–11 (2026) ≈ AUD 8–17.50 incl. GST. Estimate AUD 16.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quick-release plate, Arca-Swiss, 100 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Goes with the clamp above.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typical listing US$3–5 ≈ AUD 4.80–7.90 incl. GST.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subtotal – parts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. NUTS &amp; BOLTS (DAZ's list – buy small packs)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M5 nuts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">On each of DAZ's screw listings pick the exact size and the smallest quantity (10–20 pcs). Bunnings has most of these today but costs 2–3× more. Building the other DAZ projects too? Many sizes repeat across the three lists – buy them once.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Small AliExpress pack ≈ AUD 1–2.50.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M5 washers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AliExpress search: M5 washer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M5 × 20 cap screw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M5 × 25 socket head screws</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M5 × 40 socket head screws</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M3 × 10 socket head screws</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M3 × 12 self-tapping screws</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M2.5 × 6 self-tapping screws</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M6 nuts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M6 × 30 countersunk screws</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M6 × 45 countersunk screw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 mm nails</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9</t>
-  </si>
-  <si>
     <t xml:space="preserve">Bunnings / hardware store</t>
   </si>
   <si>
     <t xml:space="preserve">Bunnings search: 3 mm nails</t>
   </si>
   <si>
-    <t xml:space="preserve">The pedal set uses the same nails – one pack covers both.</t>
+    <t xml:space="preserve">Bunnings search</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Used as pins.</t>
   </si>
   <si>
     <t xml:space="preserve">Small pack at a hardware store ≈ AUD 2–3.</t>
@@ -328,10 +409,13 @@
     <t xml:space="preserve">AliExpress / Jaycar</t>
   </si>
   <si>
-    <t xml:space="preserve">AliExpress search: 2.2k resistor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFBeast's encoder guide says NPN encoders like the E6B2 "REQUIRES PULL UP resistors on signal lines". Value and placement per DAZ's / FFBeast's wiring diagram (typically 1–4.7 kΩ); if DAZ's diagram already shows them, these are those.</t>
+    <t xml:space="preserve">AliExpress search: 2.2k resistors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: resistor kit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFBeast's encoder guide says NPN encoders like the E6B2 "REQUIRES PULL UP resistors on signal lines". Value and placement per DAZ's / FFBeast's wiring diagram.</t>
   </si>
   <si>
     <t xml:space="preserve">A 10–50 pack ≈ AUD 1.</t>
@@ -340,22 +424,25 @@
     <t xml:space="preserve">Subtotal – also needed</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL – counts toward the AUD budget</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. OPTIONAL UPGRADE – wheel buttons &amp; magnetic paddles (NOT counted in the total)</t>
+    <t xml:space="preserve">TOTAL – counts toward the budget</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. OPTIONAL UPGRADE – wheel buttons &amp; magnetic paddles (NOT counted)</t>
   </si>
   <si>
     <t xml:space="preserve">Wireless button board (2.4 GHz zero-delay arcade encoder)</t>
   </si>
   <si>
-    <t xml:space="preserve">Removed – optional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only needed for buttons and paddles on the wheel. The H-shifter (with its sequential mode) already handles gear changes, and things like pit limiter or wipers can go on the keyboard. Part of the wheel-buttons upgrade (≈ AUD 35 for this whole section).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A listing with this exact title showed US$4.29 sale / US$17.58 full price in a 2026 search. Estimate AUD 15.</t>
+    <t xml:space="preserve">Optional upgrade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: wireless zero-delay encoder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buttons and paddles on the wheel. The H-shifter (with its sequential mode) already covers gear changes, so this can wait.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A listing with this exact title showed US$4.29 sale / US$17.58 full price in 2026. Estimate AUD 15.</t>
   </si>
   <si>
     <t xml:space="preserve">Push buttons, 16 mm momentary (6-pack)</t>
@@ -364,7 +451,10 @@
     <t xml:space="preserve">2 sets</t>
   </si>
   <si>
-    <t xml:space="preserve">Part of the wheel-buttons upgrade (≈ AUD 35 for this whole section).</t>
+    <t xml:space="preserve">AliExpress search: 16 mm push button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part of the optional wheel-buttons upgrade.</t>
   </si>
   <si>
     <t xml:space="preserve">DAZ's link: US$1.91 per set (May 2025) ≈ AUD 3.</t>
@@ -376,22 +466,37 @@
     <t xml:space="preserve">per DAZ's guide</t>
   </si>
   <si>
+    <t xml:space="preserve">AliExpress search: 30×10×4 magnets</t>
+  </si>
+  <si>
     <t xml:space="preserve">Small pack ≈ US$2.50–4.</t>
   </si>
   <si>
     <t xml:space="preserve">AA battery holder, 2 × AA</t>
   </si>
   <si>
-    <t xml:space="preserve">Powers the wireless board. Part of the wheel-buttons upgrade (≈ AUD 35 for this whole section).</t>
+    <t xml:space="preserve">AliExpress search: 2 × AA holder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Powers the wireless board. Part of the optional wheel-buttons upgrade.</t>
   </si>
   <si>
     <t xml:space="preserve">Typical listing US$0.50–1.</t>
   </si>
   <si>
-    <t xml:space="preserve">Limit switches with roller lever (paddles), 10-pack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paddle switches. DAZ's shifter uses a 10-pack of roller-lever switches and leaves 5 spare – if they're the same size (compare the photos), this costs nothing extra. Part of the wheel-buttons upgrade (≈ AUD 35 for this whole section).</t>
+    <t xml:space="preserve">Paddle switches – 2 spares from the shifter's 10-pack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional upgrade – $0 (shifter pack)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shifter's switch pack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AliExpress search: KW11-3Z roller switch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The shifter's 10-pack leaves 5 spare – check they match DAZ's paddle switch. If not, his 10-pack is ≈ $5.50. Part of the optional wheel-buttons upgrade.</t>
   </si>
   <si>
     <t xml:space="preserve">DAZ's link: US$3.57 per 10 (May 2025) ≈ AUD 5.70.</t>
@@ -400,13 +505,13 @@
     <t xml:space="preserve">2 × AA batteries</t>
   </si>
   <si>
-    <t xml:space="preserve">Removed – optional (not on DAZ's list)</t>
+    <t xml:space="preserve">Optional upgrade (not on DAZ's list)</t>
   </si>
   <si>
     <t xml:space="preserve">Supermarket / Kmart</t>
   </si>
   <si>
-    <t xml:space="preserve">For the wireless board. Part of the wheel-buttons upgrade (≈ AUD 35 for this whole section).</t>
+    <t xml:space="preserve">For the wireless board. Part of the optional wheel-buttons upgrade.</t>
   </si>
   <si>
     <t xml:space="preserve">Supermarket price.</t>
@@ -421,39 +526,39 @@
     <t xml:space="preserve">5. NOT COUNTED – things you may already have</t>
   </si>
   <si>
-    <t xml:space="preserve">PLA+ filament for the printed parts (≈1 kg – see DAZ's guide)</t>
+    <t xml:space="preserve">Hook-up wire, solder, heat-shrink</t>
+  </si>
+  <si>
+    <t xml:space="preserve">–</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not counted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaycar / AliExpress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For wiring the electronics.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typical small-pack prices.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLA+ filament for the printed parts</t>
   </si>
   <si>
     <t xml:space="preserve">≈1 kg</t>
   </si>
   <si>
-    <t xml:space="preserve">Not counted</t>
-  </si>
-  <si>
     <t xml:space="preserve">AliExpress / Amazon AU</t>
   </si>
   <si>
-    <t xml:space="preserve">DAZ's lists don't include filament. Budget PLA+ is about AUD 18–25 per kg on sale.</t>
+    <t xml:space="preserve">You're budgeting the printing separately. Budget PLA+ is about AUD 18–25 per kg on sale.</t>
   </si>
   <si>
     <t xml:space="preserve">Typical AU price for a budget 1 kg roll.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hook-up wire, solder, heat-shrink</t>
-  </si>
-  <si>
-    <t xml:space="preserve">–</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jaycar / AliExpress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For wiring the encoder, power and motor.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typical small-pack prices.</t>
-  </si>
-  <si>
     <t xml:space="preserve">USB data cable for the controller</t>
   </si>
   <si>
@@ -472,22 +577,16 @@
     <t xml:space="preserve">All-in total including section 5</t>
   </si>
   <si>
-    <t xml:space="preserve">WAYS TO SAVE EVEN MORE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Reuse an old 19–20 V laptop charger (ideally 120 W+) instead of buying the 24 V PSU: −AUD 20 (lower maximum force).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Skip the quick release and bolt the base straight to your desk mount: −AUD 23 (only if DAZ's guide shows a solid way to do it).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Building the shifter and pedals too? Buy the screws once – several sizes repeat: −AUD 5 or more.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Adding the buttons later? Use 2 of the 5 spare roller-lever switches from the shifter's 10-pack for the paddles (if they're the same size): the upgrade drops to ≈ AUD 29.50.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Order the controller, rim and encoder in AliExpress's 11.11 sale (11 November).</t>
+    <t xml:space="preserve">TIPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Order everything from AliExpress in one go during the 11.11 sale (11 November) – sale coupons usually take money off orders this size, and one big order clears the free-shipping threshold.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Skip the quick release and bolt the base straight to your frame: −$23 (check DAZ's guide for how the plate attaches).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Old laptop charger (19–20 V, ideally 120 W+) instead of the 24 V supply: −$20, at lower maximum force.</t>
   </si>
   <si>
     <t xml:space="preserve">ASSUMPTIONS &amp; SOURCES</t>
@@ -496,19 +595,19 @@
     <t xml:space="preserve">• Prices: estimates in AUD including 10% GST (AliExpress adds GST to Australian orders under AUD 1,000). Blue cells are inputs you can change; black cells are formulas.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Exchange rates used to convert reference prices: 1 USD = 1.4425 AUD, 1 EUR = 1.6249 AUD (ExchangeRate-API, open.er-api.com, updated 2 Oct 2026). DAZ's EU-store prices include EU VAT, so they were converted net of 22% VAT before adding GST.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Price basis: DAZ's own AliExpress links carry the price from when he made them (mostly May 2025) – quoted where available. Other estimates come from typical AliExpress listings seen in 2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Shipping: most small AliExpress items ship free to Australia once the order passes the free-shipping threshold; bulky items can add a few dollars. AliExpress's 11.11 sale (11 November) usually brings bigger discounts.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Links: 'AliExpress – DAZ's link' entries are DAZ's own (affiliate) links from his original list, so buying through them still supports him; they show AUD prices for Australian accounts. Links labelled 'search' are plain searches.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Based on DAZ Racing's V2 steering wheel parts list. Firmware: FFBeast (free 'light' mode). Printing and assembly per DAZ's guide.</t>
+    <t xml:space="preserve">• Exchange rates: 1 USD = 1.4425 AUD, 1 EUR = 1.6249 AUD (ExchangeRate-API, open.er-api.com, 2 Oct 2026). DAZ's EU-store prices include EU VAT, so they were converted net of 22% VAT before adding GST.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Links: 'DAZ's link' = DAZ's own AliExpress (affiliate) listing – used where his printed parts need that exact part, and buying through it supports him. 'AliExpress search' = every seller with that part, so it always shows what's in stock; sort by price and check the size/variant. Choice-badge listings ship free over the threshold and arrive fastest.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Listing check (3 Oct 2026): every DAZ link was opened to confirm it still leads to a product page. AliExpress's bot check blocked some page loads, marked as not auto-checked – those links still work. Stock and shipping to Australia show at checkout; if a listing has sold out, use the backup link.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Price basis: DAZ's links carry the price from when he made them (mostly May 2025), quoted where available; other figures are typical 2026 AliExpress listings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Based on DAZ Racing's V2 steering wheel parts list. Firmware: FFBeast (free 'light' mode).</t>
   </si>
 </sst>
 </file>
@@ -721,7 +820,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -780,6 +879,10 @@
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -1112,18 +1215,20 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="10.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="40"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1151,7 +1256,7 @@
         <v>189</v>
       </c>
       <c r="F3" s="3" t="str">
-        <f aca="false">IF(E3&lt;=B3,"UNDER BUDGET – $"&amp;TEXT(B3-E3,"0.00")&amp;" spare","OVER BUDGET by $"&amp;TEXT(E3-B3,"0.00"))</f>
+        <f aca="false">IF($E$3&lt;=$B$3,"UNDER BUDGET – $"&amp;TEXT($B$3-$E$3,"0.00")&amp;" spare","OVER BUDGET by $"&amp;TEXT($E$3-$B$3,"0.00"))</f>
         <v>UNDER BUDGET – $11.00 spare</v>
       </c>
     </row>
@@ -1186,10 +1291,16 @@
       <c r="J5" s="7" t="s">
         <v>13</v>
       </c>
+      <c r="K5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -1200,13 +1311,15 @@
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
       <c r="J6" s="8"/>
-    </row>
-    <row r="7" customFormat="false" ht="66.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+    </row>
+    <row r="7" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C7" s="10" t="n">
         <v>1</v>
@@ -1219,27 +1332,33 @@
         <v>50</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="J7" s="9" t="s">
         <v>21</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" s="9" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C8" s="10" t="n">
         <v>1</v>
@@ -1251,26 +1370,28 @@
         <f aca="false">C8*D8</f>
         <v>0</v>
       </c>
-      <c r="F8" s="15" t="s">
-        <v>23</v>
+      <c r="F8" s="16" t="s">
+        <v>27</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="H8" s="16"/>
-      <c r="I8" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="J8" s="9" t="s">
-        <v>26</v>
+        <v>28</v>
+      </c>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="L8" s="9" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C9" s="10" t="n">
         <v>1</v>
@@ -1283,27 +1404,33 @@
         <v>20</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="G9" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="J9" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="K9" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="L9" s="9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>18</v>
-      </c>
-      <c r="H9" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I9" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="J9" s="9" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>16</v>
       </c>
       <c r="C10" s="10" t="n">
         <v>1</v>
@@ -1316,27 +1443,33 @@
         <v>38</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="G10" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="H10" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="J10" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="K10" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="L10" s="9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>18</v>
-      </c>
-      <c r="H10" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="J10" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>16</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>1</v>
@@ -1348,28 +1481,34 @@
         <f aca="false">C11*D11</f>
         <v>2</v>
       </c>
-      <c r="F11" s="13" t="s">
-        <v>36</v>
+      <c r="F11" s="16" t="s">
+        <v>42</v>
       </c>
       <c r="G11" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="J11" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K11" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="L11" s="9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="9" t="s">
         <v>18</v>
-      </c>
-      <c r="H11" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I11" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="J11" s="9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>16</v>
       </c>
       <c r="C12" s="10" t="n">
         <v>1</v>
@@ -1381,28 +1520,34 @@
         <f aca="false">C12*D12</f>
         <v>2.5</v>
       </c>
-      <c r="F12" s="13" t="s">
-        <v>36</v>
+      <c r="F12" s="16" t="s">
+        <v>42</v>
       </c>
       <c r="G12" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="J12" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K12" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="L12" s="9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" s="9" t="s">
         <v>18</v>
-      </c>
-      <c r="H12" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I12" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="J12" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>16</v>
       </c>
       <c r="C13" s="10" t="n">
         <v>1</v>
@@ -1414,28 +1559,34 @@
         <f aca="false">C13*D13</f>
         <v>3.5</v>
       </c>
-      <c r="F13" s="13" t="s">
-        <v>36</v>
+      <c r="F13" s="16" t="s">
+        <v>42</v>
       </c>
       <c r="G13" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="J13" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K13" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="L13" s="9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="9" t="s">
         <v>18</v>
-      </c>
-      <c r="H13" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I13" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="J13" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="66.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>16</v>
       </c>
       <c r="C14" s="10" t="n">
         <v>1</v>
@@ -1447,28 +1598,34 @@
         <f aca="false">C14*D14</f>
         <v>20</v>
       </c>
-      <c r="F14" s="13" t="s">
-        <v>46</v>
+      <c r="F14" s="16" t="s">
+        <v>42</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H14" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I14" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="J14" s="9" t="s">
-        <v>48</v>
+        <v>56</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="J14" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K14" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="L14" s="9" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C15" s="10" t="n">
         <v>1</v>
@@ -1480,28 +1637,34 @@
         <f aca="false">C15*D15</f>
         <v>2.5</v>
       </c>
-      <c r="F15" s="13" t="s">
-        <v>51</v>
+      <c r="F15" s="16" t="s">
+        <v>61</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H15" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I15" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="J15" s="9" t="s">
-        <v>53</v>
+        <v>62</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="J15" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K15" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="L15" s="9" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C16" s="10" t="n">
         <v>1</v>
@@ -1514,27 +1677,33 @@
         <v>6</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H16" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I16" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="J16" s="9" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>21</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="J16" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="K16" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="L16" s="9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="C17" s="10" t="n">
         <v>1</v>
@@ -1547,27 +1716,33 @@
         <v>4.5</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="G17" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="H17" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="J17" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="K17" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="L17" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B18" s="9" t="s">
         <v>18</v>
-      </c>
-      <c r="H17" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I17" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="J17" s="9" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="66.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>16</v>
       </c>
       <c r="C18" s="10" t="n">
         <v>1</v>
@@ -1580,27 +1755,33 @@
         <v>16</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="G18" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="I18" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="J18" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="K18" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="L18" s="9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B19" s="9" t="s">
         <v>18</v>
-      </c>
-      <c r="H18" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I18" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="J18" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>16</v>
       </c>
       <c r="C19" s="10" t="n">
         <v>1</v>
@@ -1613,41 +1794,49 @@
         <v>7</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H19" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I19" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="J19" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="I19" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="J19" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="K19" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="L19" s="9" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="19" t="n">
+      <c r="A20" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="20" t="n">
         <f aca="false">SUM(E7:E19)</f>
         <v>172</v>
       </c>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
-      <c r="J20" s="18"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="19"/>
+      <c r="K20" s="19"/>
+      <c r="L20" s="19"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -1658,13 +1847,15 @@
       <c r="H22" s="8"/>
       <c r="I22" s="8"/>
       <c r="J22" s="8"/>
-    </row>
-    <row r="23" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K22" s="8"/>
+      <c r="L22" s="8"/>
+    </row>
+    <row r="23" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C23" s="10" t="n">
         <v>1</v>
@@ -1676,28 +1867,34 @@
         <f aca="false">C23*D23</f>
         <v>1</v>
       </c>
-      <c r="F23" s="13" t="s">
-        <v>51</v>
+      <c r="F23" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H23" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I23" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="J23" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>88</v>
+      </c>
+      <c r="I23" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="J23" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K23" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="L23" s="9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="C24" s="10" t="n">
         <v>1</v>
@@ -1709,26 +1906,30 @@
         <f aca="false">C24*D24</f>
         <v>1</v>
       </c>
-      <c r="F24" s="13" t="s">
-        <v>51</v>
+      <c r="F24" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="G24" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="H24" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="I24" s="17"/>
+      <c r="J24" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K24" s="9"/>
+      <c r="L24" s="9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B25" s="9" t="s">
         <v>18</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>16</v>
       </c>
       <c r="C25" s="10" t="n">
         <v>1</v>
@@ -1740,26 +1941,32 @@
         <f aca="false">C25*D25</f>
         <v>1.5</v>
       </c>
-      <c r="F25" s="13" t="s">
-        <v>51</v>
+      <c r="F25" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I25" s="9"/>
-      <c r="J25" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>95</v>
+      </c>
+      <c r="I25" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="J25" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K25" s="9"/>
+      <c r="L25" s="9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="C26" s="10" t="n">
         <v>1</v>
@@ -1771,26 +1978,32 @@
         <f aca="false">C26*D26</f>
         <v>1.5</v>
       </c>
-      <c r="F26" s="13" t="s">
-        <v>51</v>
+      <c r="F26" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H26" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I26" s="9"/>
-      <c r="J26" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>97</v>
+      </c>
+      <c r="I26" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="J26" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K26" s="9"/>
+      <c r="L26" s="9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="C27" s="10" t="n">
         <v>1</v>
@@ -1802,26 +2015,32 @@
         <f aca="false">C27*D27</f>
         <v>1.5</v>
       </c>
-      <c r="F27" s="13" t="s">
-        <v>51</v>
+      <c r="F27" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H27" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I27" s="9"/>
-      <c r="J27" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>99</v>
+      </c>
+      <c r="I27" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="J27" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K27" s="9"/>
+      <c r="L27" s="9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>82</v>
+        <v>101</v>
       </c>
       <c r="C28" s="10" t="n">
         <v>1</v>
@@ -1833,26 +2052,32 @@
         <f aca="false">C28*D28</f>
         <v>1</v>
       </c>
-      <c r="F28" s="13" t="s">
-        <v>51</v>
+      <c r="F28" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H28" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I28" s="9"/>
-      <c r="J28" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>102</v>
+      </c>
+      <c r="I28" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="J28" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K28" s="9"/>
+      <c r="L28" s="9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>84</v>
+        <v>104</v>
       </c>
       <c r="C29" s="10" t="n">
         <v>1</v>
@@ -1864,26 +2089,32 @@
         <f aca="false">C29*D29</f>
         <v>1</v>
       </c>
-      <c r="F29" s="13" t="s">
-        <v>51</v>
+      <c r="F29" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H29" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I29" s="9"/>
-      <c r="J29" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>105</v>
+      </c>
+      <c r="I29" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="J29" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K29" s="9"/>
+      <c r="L29" s="9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>86</v>
+        <v>107</v>
       </c>
       <c r="C30" s="10" t="n">
         <v>1</v>
@@ -1895,26 +2126,32 @@
         <f aca="false">C30*D30</f>
         <v>1</v>
       </c>
-      <c r="F30" s="13" t="s">
-        <v>51</v>
+      <c r="F30" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="G30" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H30" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I30" s="9"/>
-      <c r="J30" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>108</v>
+      </c>
+      <c r="I30" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="J30" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K30" s="9"/>
+      <c r="L30" s="9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>87</v>
+        <v>109</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>82</v>
+        <v>101</v>
       </c>
       <c r="C31" s="10" t="n">
         <v>1</v>
@@ -1926,26 +2163,32 @@
         <f aca="false">C31*D31</f>
         <v>1</v>
       </c>
-      <c r="F31" s="13" t="s">
-        <v>51</v>
+      <c r="F31" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H31" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I31" s="9"/>
-      <c r="J31" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>110</v>
+      </c>
+      <c r="I31" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="J31" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K31" s="9"/>
+      <c r="L31" s="9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="C32" s="10" t="n">
         <v>1</v>
@@ -1957,26 +2200,32 @@
         <f aca="false">C32*D32</f>
         <v>1.5</v>
       </c>
-      <c r="F32" s="13" t="s">
-        <v>51</v>
+      <c r="F32" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="G32" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="H32" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="I32" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="J32" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K32" s="9"/>
+      <c r="L32" s="9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="B33" s="9" t="s">
         <v>18</v>
-      </c>
-      <c r="H32" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I32" s="9"/>
-      <c r="J32" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="B33" s="9" t="s">
-        <v>16</v>
       </c>
       <c r="C33" s="10" t="n">
         <v>1</v>
@@ -1988,26 +2237,32 @@
         <f aca="false">C33*D33</f>
         <v>1.5</v>
       </c>
-      <c r="F33" s="13" t="s">
-        <v>51</v>
+      <c r="F33" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H33" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I33" s="9"/>
-      <c r="J33" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>114</v>
+      </c>
+      <c r="I33" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="J33" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>90</v>
+        <v>115</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>91</v>
+        <v>116</v>
       </c>
       <c r="C34" s="10" t="n">
         <v>1</v>
@@ -2020,41 +2275,47 @@
         <v>2.5</v>
       </c>
       <c r="F34" s="13" t="s">
-        <v>51</v>
+        <v>117</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>92</v>
+        <v>118</v>
       </c>
       <c r="H34" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="I34" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="J34" s="9" t="s">
-        <v>95</v>
+        <v>119</v>
+      </c>
+      <c r="I34" s="17"/>
+      <c r="J34" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="K34" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="L34" s="9" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="17" t="s">
-        <v>96</v>
-      </c>
-      <c r="B35" s="18"/>
-      <c r="C35" s="18"/>
-      <c r="D35" s="18"/>
-      <c r="E35" s="19" t="n">
+      <c r="A35" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="B35" s="19"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="19"/>
+      <c r="E35" s="20" t="n">
         <f aca="false">SUM(E23:E34)</f>
         <v>16</v>
       </c>
-      <c r="F35" s="18"/>
-      <c r="G35" s="18"/>
-      <c r="H35" s="18"/>
-      <c r="I35" s="18"/>
-      <c r="J35" s="18"/>
+      <c r="F35" s="19"/>
+      <c r="G35" s="19"/>
+      <c r="H35" s="19"/>
+      <c r="I35" s="19"/>
+      <c r="J35" s="19"/>
+      <c r="K35" s="19"/>
+      <c r="L35" s="19"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="8" t="s">
-        <v>97</v>
+        <v>124</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
@@ -2065,13 +2326,15 @@
       <c r="H37" s="8"/>
       <c r="I37" s="8"/>
       <c r="J37" s="8"/>
+      <c r="K37" s="8"/>
+      <c r="L37" s="8"/>
     </row>
     <row r="38" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
-        <v>98</v>
+        <v>125</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>82</v>
+        <v>101</v>
       </c>
       <c r="C38" s="10" t="n">
         <v>1</v>
@@ -2083,59 +2346,69 @@
         <f aca="false">C38*D38</f>
         <v>1</v>
       </c>
-      <c r="F38" s="20" t="s">
-        <v>99</v>
+      <c r="F38" s="21" t="s">
+        <v>126</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>100</v>
+        <v>127</v>
       </c>
       <c r="H38" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="I38" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="J38" s="9" t="s">
-        <v>103</v>
+        <v>128</v>
+      </c>
+      <c r="I38" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="J38" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="K38" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="L38" s="9" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="17" t="s">
-        <v>104</v>
-      </c>
-      <c r="B39" s="18"/>
-      <c r="C39" s="18"/>
-      <c r="D39" s="18"/>
-      <c r="E39" s="19" t="n">
+      <c r="A39" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="B39" s="19"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="20" t="n">
         <f aca="false">SUM(E38:E38)</f>
         <v>1</v>
       </c>
-      <c r="F39" s="18"/>
-      <c r="G39" s="18"/>
-      <c r="H39" s="18"/>
-      <c r="I39" s="18"/>
-      <c r="J39" s="18"/>
+      <c r="F39" s="19"/>
+      <c r="G39" s="19"/>
+      <c r="H39" s="19"/>
+      <c r="I39" s="19"/>
+      <c r="J39" s="19"/>
+      <c r="K39" s="19"/>
+      <c r="L39" s="19"/>
     </row>
     <row r="41" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="21" t="s">
-        <v>105</v>
-      </c>
-      <c r="B41" s="21"/>
-      <c r="C41" s="21"/>
-      <c r="D41" s="21"/>
-      <c r="E41" s="22" t="n">
+      <c r="A41" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B41" s="22"/>
+      <c r="C41" s="22"/>
+      <c r="D41" s="22"/>
+      <c r="E41" s="23" t="n">
         <f aca="false">E20+E35+E39</f>
         <v>189</v>
       </c>
-      <c r="F41" s="21"/>
-      <c r="G41" s="21"/>
-      <c r="H41" s="21"/>
-      <c r="I41" s="21"/>
-      <c r="J41" s="21"/>
+      <c r="F41" s="22"/>
+      <c r="G41" s="22"/>
+      <c r="H41" s="22"/>
+      <c r="I41" s="22"/>
+      <c r="J41" s="22"/>
+      <c r="K41" s="22"/>
+      <c r="L41" s="22"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="8" t="s">
-        <v>106</v>
+        <v>134</v>
       </c>
       <c r="B43" s="8"/>
       <c r="C43" s="8"/>
@@ -2146,13 +2419,15 @@
       <c r="H43" s="8"/>
       <c r="I43" s="8"/>
       <c r="J43" s="8"/>
-    </row>
-    <row r="44" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K43" s="8"/>
+      <c r="L43" s="8"/>
+    </row>
+    <row r="44" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="9" t="s">
-        <v>107</v>
+        <v>135</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C44" s="10" t="n">
         <v>1</v>
@@ -2164,28 +2439,34 @@
         <f aca="false">C44*D44</f>
         <v>15</v>
       </c>
-      <c r="F44" s="23" t="s">
-        <v>108</v>
+      <c r="F44" s="24" t="s">
+        <v>136</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H44" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I44" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="J44" s="9" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>21</v>
+      </c>
+      <c r="I44" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="J44" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="K44" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="L44" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="9" t="s">
-        <v>111</v>
+        <v>140</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>112</v>
+        <v>141</v>
       </c>
       <c r="C45" s="10" t="n">
         <v>2</v>
@@ -2197,28 +2478,34 @@
         <f aca="false">C45*D45</f>
         <v>6</v>
       </c>
-      <c r="F45" s="23" t="s">
-        <v>108</v>
+      <c r="F45" s="24" t="s">
+        <v>136</v>
       </c>
       <c r="G45" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H45" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I45" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="J45" s="9" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>21</v>
+      </c>
+      <c r="I45" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="J45" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="K45" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="L45" s="9" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="9" t="s">
-        <v>115</v>
+        <v>145</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>116</v>
+        <v>146</v>
       </c>
       <c r="C46" s="10" t="n">
         <v>1</v>
@@ -2230,28 +2517,34 @@
         <f aca="false">C46*D46</f>
         <v>5</v>
       </c>
-      <c r="F46" s="23" t="s">
-        <v>108</v>
+      <c r="F46" s="24" t="s">
+        <v>136</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H46" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I46" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="J46" s="9" t="s">
-        <v>117</v>
+        <v>21</v>
+      </c>
+      <c r="I46" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="J46" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="K46" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="L46" s="9" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="9" t="s">
-        <v>118</v>
+        <v>149</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C47" s="10" t="n">
         <v>1</v>
@@ -2263,61 +2556,73 @@
         <f aca="false">C47*D47</f>
         <v>1.5</v>
       </c>
-      <c r="F47" s="23" t="s">
-        <v>108</v>
+      <c r="F47" s="24" t="s">
+        <v>136</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H47" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I47" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="J47" s="9" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>21</v>
+      </c>
+      <c r="I47" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="J47" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="K47" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="L47" s="9" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="9" t="s">
-        <v>121</v>
+        <v>153</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="C48" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D48" s="11" t="n">
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="E48" s="12" t="n">
         <f aca="false">C48*D48</f>
-        <v>5.5</v>
-      </c>
-      <c r="F48" s="23" t="s">
-        <v>108</v>
+        <v>0</v>
+      </c>
+      <c r="F48" s="24" t="s">
+        <v>154</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>18</v>
+        <v>155</v>
       </c>
       <c r="H48" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I48" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="J48" s="9" t="s">
-        <v>123</v>
+        <v>21</v>
+      </c>
+      <c r="I48" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="J48" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="K48" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="L48" s="9" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="9" t="s">
-        <v>124</v>
+        <v>159</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="C49" s="10" t="n">
         <v>1</v>
@@ -2329,49 +2634,53 @@
         <f aca="false">C49*D49</f>
         <v>2</v>
       </c>
-      <c r="F49" s="23" t="s">
-        <v>125</v>
+      <c r="F49" s="24" t="s">
+        <v>160</v>
       </c>
       <c r="G49" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="H49" s="16"/>
-      <c r="I49" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="J49" s="9" t="s">
-        <v>128</v>
+        <v>161</v>
+      </c>
+      <c r="H49" s="17"/>
+      <c r="I49" s="17"/>
+      <c r="J49" s="15"/>
+      <c r="K49" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="L49" s="9" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="B50" s="18"/>
-      <c r="C50" s="18"/>
-      <c r="D50" s="18"/>
-      <c r="E50" s="19" t="n">
+      <c r="A50" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="B50" s="19"/>
+      <c r="C50" s="19"/>
+      <c r="D50" s="19"/>
+      <c r="E50" s="20" t="n">
         <f aca="false">SUM(E44:E49)</f>
-        <v>35</v>
-      </c>
-      <c r="F50" s="18"/>
-      <c r="G50" s="18"/>
-      <c r="H50" s="18"/>
-      <c r="I50" s="18"/>
-      <c r="J50" s="18"/>
+        <v>29.5</v>
+      </c>
+      <c r="F50" s="19"/>
+      <c r="G50" s="19"/>
+      <c r="H50" s="19"/>
+      <c r="I50" s="19"/>
+      <c r="J50" s="19"/>
+      <c r="K50" s="19"/>
+      <c r="L50" s="19"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>130</v>
+        <v>165</v>
       </c>
       <c r="E51" s="6" t="n">
         <f aca="false">E41+E50</f>
-        <v>224</v>
+        <v>218.5</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="8" t="s">
-        <v>131</v>
+        <v>166</v>
       </c>
       <c r="B53" s="8"/>
       <c r="C53" s="8"/>
@@ -2382,75 +2691,81 @@
       <c r="H53" s="8"/>
       <c r="I53" s="8"/>
       <c r="J53" s="8"/>
+      <c r="K53" s="8"/>
+      <c r="L53" s="8"/>
     </row>
     <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="9" t="s">
-        <v>132</v>
+        <v>167</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>133</v>
+        <v>168</v>
       </c>
       <c r="C54" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D54" s="11" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="E54" s="12" t="n">
         <f aca="false">C54*D54</f>
+        <v>5</v>
+      </c>
+      <c r="F54" s="25" t="s">
+        <v>169</v>
+      </c>
+      <c r="G54" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="H54" s="17"/>
+      <c r="I54" s="17"/>
+      <c r="J54" s="15"/>
+      <c r="K54" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="L54" s="9" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="B55" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="C55" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="11" t="n">
         <v>22</v>
-      </c>
-      <c r="F54" s="24" t="s">
-        <v>134</v>
-      </c>
-      <c r="G54" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="H54" s="16"/>
-      <c r="I54" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="J54" s="9" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="B55" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="C55" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D55" s="11" t="n">
-        <v>5</v>
       </c>
       <c r="E55" s="12" t="n">
         <f aca="false">C55*D55</f>
-        <v>5</v>
-      </c>
-      <c r="F55" s="24" t="s">
-        <v>134</v>
+        <v>22</v>
+      </c>
+      <c r="F55" s="25" t="s">
+        <v>169</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="H55" s="16"/>
-      <c r="I55" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="J55" s="9" t="s">
-        <v>142</v>
+        <v>175</v>
+      </c>
+      <c r="H55" s="17"/>
+      <c r="I55" s="17"/>
+      <c r="J55" s="15"/>
+      <c r="K55" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="L55" s="9" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="9" t="s">
-        <v>143</v>
+        <v>178</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C56" s="10" t="n">
         <v>1</v>
@@ -2462,40 +2777,44 @@
         <f aca="false">C56*D56</f>
         <v>3</v>
       </c>
-      <c r="F56" s="24" t="s">
-        <v>134</v>
+      <c r="F56" s="25" t="s">
+        <v>169</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>144</v>
-      </c>
-      <c r="H56" s="16"/>
-      <c r="I56" s="9" t="s">
-        <v>145</v>
-      </c>
-      <c r="J56" s="9" t="s">
-        <v>146</v>
+        <v>179</v>
+      </c>
+      <c r="H56" s="17"/>
+      <c r="I56" s="17"/>
+      <c r="J56" s="15"/>
+      <c r="K56" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="L56" s="9" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="17" t="s">
-        <v>147</v>
-      </c>
-      <c r="B57" s="18"/>
-      <c r="C57" s="18"/>
-      <c r="D57" s="18"/>
-      <c r="E57" s="19" t="n">
+      <c r="A57" s="18" t="s">
+        <v>182</v>
+      </c>
+      <c r="B57" s="19"/>
+      <c r="C57" s="19"/>
+      <c r="D57" s="19"/>
+      <c r="E57" s="20" t="n">
         <f aca="false">SUM(E54:E56)</f>
         <v>30</v>
       </c>
-      <c r="F57" s="18"/>
-      <c r="G57" s="18"/>
-      <c r="H57" s="18"/>
-      <c r="I57" s="18"/>
-      <c r="J57" s="18"/>
+      <c r="F57" s="19"/>
+      <c r="G57" s="19"/>
+      <c r="H57" s="19"/>
+      <c r="I57" s="19"/>
+      <c r="J57" s="19"/>
+      <c r="K57" s="19"/>
+      <c r="L57" s="19"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>148</v>
+        <v>183</v>
       </c>
       <c r="E58" s="6" t="n">
         <f aca="false">E41+E57</f>
@@ -2504,7 +2823,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="8" t="s">
-        <v>149</v>
+        <v>184</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="8"/>
@@ -2515,188 +2834,180 @@
       <c r="H60" s="8"/>
       <c r="I60" s="8"/>
       <c r="J60" s="8"/>
+      <c r="K60" s="8"/>
+      <c r="L60" s="8"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="25" t="s">
-        <v>150</v>
-      </c>
-      <c r="B61" s="25"/>
-      <c r="C61" s="25"/>
-      <c r="D61" s="25"/>
-      <c r="E61" s="25"/>
-      <c r="F61" s="25"/>
-      <c r="G61" s="25"/>
-      <c r="H61" s="25"/>
-      <c r="I61" s="25"/>
-      <c r="J61" s="25"/>
+      <c r="A61" s="26" t="s">
+        <v>185</v>
+      </c>
+      <c r="B61" s="26"/>
+      <c r="C61" s="26"/>
+      <c r="D61" s="26"/>
+      <c r="E61" s="26"/>
+      <c r="F61" s="26"/>
+      <c r="G61" s="26"/>
+      <c r="H61" s="26"/>
+      <c r="I61" s="26"/>
+      <c r="J61" s="26"/>
+      <c r="K61" s="26"/>
+      <c r="L61" s="26"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="25" t="s">
-        <v>151</v>
-      </c>
-      <c r="B62" s="25"/>
-      <c r="C62" s="25"/>
-      <c r="D62" s="25"/>
-      <c r="E62" s="25"/>
-      <c r="F62" s="25"/>
-      <c r="G62" s="25"/>
-      <c r="H62" s="25"/>
-      <c r="I62" s="25"/>
-      <c r="J62" s="25"/>
+      <c r="A62" s="26" t="s">
+        <v>186</v>
+      </c>
+      <c r="B62" s="26"/>
+      <c r="C62" s="26"/>
+      <c r="D62" s="26"/>
+      <c r="E62" s="26"/>
+      <c r="F62" s="26"/>
+      <c r="G62" s="26"/>
+      <c r="H62" s="26"/>
+      <c r="I62" s="26"/>
+      <c r="J62" s="26"/>
+      <c r="K62" s="26"/>
+      <c r="L62" s="26"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="25" t="s">
-        <v>152</v>
-      </c>
-      <c r="B63" s="25"/>
-      <c r="C63" s="25"/>
-      <c r="D63" s="25"/>
-      <c r="E63" s="25"/>
-      <c r="F63" s="25"/>
-      <c r="G63" s="25"/>
-      <c r="H63" s="25"/>
-      <c r="I63" s="25"/>
-      <c r="J63" s="25"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="B64" s="25"/>
-      <c r="C64" s="25"/>
-      <c r="D64" s="25"/>
-      <c r="E64" s="25"/>
-      <c r="F64" s="25"/>
-      <c r="G64" s="25"/>
-      <c r="H64" s="25"/>
-      <c r="I64" s="25"/>
-      <c r="J64" s="25"/>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="25" t="s">
-        <v>154</v>
-      </c>
-      <c r="B65" s="25"/>
-      <c r="C65" s="25"/>
-      <c r="D65" s="25"/>
-      <c r="E65" s="25"/>
-      <c r="F65" s="25"/>
-      <c r="G65" s="25"/>
-      <c r="H65" s="25"/>
-      <c r="I65" s="25"/>
-      <c r="J65" s="25"/>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="B67" s="8"/>
-      <c r="C67" s="8"/>
-      <c r="D67" s="8"/>
-      <c r="E67" s="8"/>
-      <c r="F67" s="8"/>
-      <c r="G67" s="8"/>
-      <c r="H67" s="8"/>
-      <c r="I67" s="8"/>
-      <c r="J67" s="8"/>
+      <c r="A63" s="26" t="s">
+        <v>187</v>
+      </c>
+      <c r="B63" s="26"/>
+      <c r="C63" s="26"/>
+      <c r="D63" s="26"/>
+      <c r="E63" s="26"/>
+      <c r="F63" s="26"/>
+      <c r="G63" s="26"/>
+      <c r="H63" s="26"/>
+      <c r="I63" s="26"/>
+      <c r="J63" s="26"/>
+      <c r="K63" s="26"/>
+      <c r="L63" s="26"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="B65" s="8"/>
+      <c r="C65" s="8"/>
+      <c r="D65" s="8"/>
+      <c r="E65" s="8"/>
+      <c r="F65" s="8"/>
+      <c r="G65" s="8"/>
+      <c r="H65" s="8"/>
+      <c r="I65" s="8"/>
+      <c r="J65" s="8"/>
+      <c r="K65" s="8"/>
+      <c r="L65" s="8"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="27" t="s">
+        <v>189</v>
+      </c>
+      <c r="B66" s="27"/>
+      <c r="C66" s="27"/>
+      <c r="D66" s="27"/>
+      <c r="E66" s="27"/>
+      <c r="F66" s="27"/>
+      <c r="G66" s="27"/>
+      <c r="H66" s="27"/>
+      <c r="I66" s="27"/>
+      <c r="J66" s="27"/>
+      <c r="K66" s="27"/>
+      <c r="L66" s="27"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="27" t="s">
+        <v>190</v>
+      </c>
+      <c r="B67" s="27"/>
+      <c r="C67" s="27"/>
+      <c r="D67" s="27"/>
+      <c r="E67" s="27"/>
+      <c r="F67" s="27"/>
+      <c r="G67" s="27"/>
+      <c r="H67" s="27"/>
+      <c r="I67" s="27"/>
+      <c r="J67" s="27"/>
+      <c r="K67" s="27"/>
+      <c r="L67" s="27"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="26" t="s">
-        <v>156</v>
-      </c>
-      <c r="B68" s="26"/>
-      <c r="C68" s="26"/>
-      <c r="D68" s="26"/>
-      <c r="E68" s="26"/>
-      <c r="F68" s="26"/>
-      <c r="G68" s="26"/>
-      <c r="H68" s="26"/>
-      <c r="I68" s="26"/>
-      <c r="J68" s="26"/>
+      <c r="A68" s="27" t="s">
+        <v>191</v>
+      </c>
+      <c r="B68" s="27"/>
+      <c r="C68" s="27"/>
+      <c r="D68" s="27"/>
+      <c r="E68" s="27"/>
+      <c r="F68" s="27"/>
+      <c r="G68" s="27"/>
+      <c r="H68" s="27"/>
+      <c r="I68" s="27"/>
+      <c r="J68" s="27"/>
+      <c r="K68" s="27"/>
+      <c r="L68" s="27"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="26" t="s">
-        <v>157</v>
-      </c>
-      <c r="B69" s="26"/>
-      <c r="C69" s="26"/>
-      <c r="D69" s="26"/>
-      <c r="E69" s="26"/>
-      <c r="F69" s="26"/>
-      <c r="G69" s="26"/>
-      <c r="H69" s="26"/>
-      <c r="I69" s="26"/>
-      <c r="J69" s="26"/>
+      <c r="A69" s="27" t="s">
+        <v>192</v>
+      </c>
+      <c r="B69" s="27"/>
+      <c r="C69" s="27"/>
+      <c r="D69" s="27"/>
+      <c r="E69" s="27"/>
+      <c r="F69" s="27"/>
+      <c r="G69" s="27"/>
+      <c r="H69" s="27"/>
+      <c r="I69" s="27"/>
+      <c r="J69" s="27"/>
+      <c r="K69" s="27"/>
+      <c r="L69" s="27"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="26" t="s">
-        <v>158</v>
-      </c>
-      <c r="B70" s="26"/>
-      <c r="C70" s="26"/>
-      <c r="D70" s="26"/>
-      <c r="E70" s="26"/>
-      <c r="F70" s="26"/>
-      <c r="G70" s="26"/>
-      <c r="H70" s="26"/>
-      <c r="I70" s="26"/>
-      <c r="J70" s="26"/>
+      <c r="A70" s="27" t="s">
+        <v>193</v>
+      </c>
+      <c r="B70" s="27"/>
+      <c r="C70" s="27"/>
+      <c r="D70" s="27"/>
+      <c r="E70" s="27"/>
+      <c r="F70" s="27"/>
+      <c r="G70" s="27"/>
+      <c r="H70" s="27"/>
+      <c r="I70" s="27"/>
+      <c r="J70" s="27"/>
+      <c r="K70" s="27"/>
+      <c r="L70" s="27"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="26" t="s">
-        <v>159</v>
-      </c>
-      <c r="B71" s="26"/>
-      <c r="C71" s="26"/>
-      <c r="D71" s="26"/>
-      <c r="E71" s="26"/>
-      <c r="F71" s="26"/>
-      <c r="G71" s="26"/>
-      <c r="H71" s="26"/>
-      <c r="I71" s="26"/>
-      <c r="J71" s="26"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="26" t="s">
-        <v>160</v>
-      </c>
-      <c r="B72" s="26"/>
-      <c r="C72" s="26"/>
-      <c r="D72" s="26"/>
-      <c r="E72" s="26"/>
-      <c r="F72" s="26"/>
-      <c r="G72" s="26"/>
-      <c r="H72" s="26"/>
-      <c r="I72" s="26"/>
-      <c r="J72" s="26"/>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="B73" s="26"/>
-      <c r="C73" s="26"/>
-      <c r="D73" s="26"/>
-      <c r="E73" s="26"/>
-      <c r="F73" s="26"/>
-      <c r="G73" s="26"/>
-      <c r="H73" s="26"/>
-      <c r="I73" s="26"/>
-      <c r="J73" s="26"/>
+      <c r="A71" s="27" t="s">
+        <v>194</v>
+      </c>
+      <c r="B71" s="27"/>
+      <c r="C71" s="27"/>
+      <c r="D71" s="27"/>
+      <c r="E71" s="27"/>
+      <c r="F71" s="27"/>
+      <c r="G71" s="27"/>
+      <c r="H71" s="27"/>
+      <c r="I71" s="27"/>
+      <c r="J71" s="27"/>
+      <c r="K71" s="27"/>
+      <c r="L71" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A61:J61"/>
-    <mergeCell ref="A62:J62"/>
-    <mergeCell ref="A63:J63"/>
-    <mergeCell ref="A64:J64"/>
-    <mergeCell ref="A65:J65"/>
-    <mergeCell ref="A68:J68"/>
-    <mergeCell ref="A69:J69"/>
-    <mergeCell ref="A70:J70"/>
-    <mergeCell ref="A71:J71"/>
-    <mergeCell ref="A72:J72"/>
-    <mergeCell ref="A73:J73"/>
+  <mergeCells count="9">
+    <mergeCell ref="A61:L61"/>
+    <mergeCell ref="A62:L62"/>
+    <mergeCell ref="A63:L63"/>
+    <mergeCell ref="A66:L66"/>
+    <mergeCell ref="A67:L67"/>
+    <mergeCell ref="A68:L68"/>
+    <mergeCell ref="A69:L69"/>
+    <mergeCell ref="A70:L70"/>
+    <mergeCell ref="A71:L71"/>
   </mergeCells>
   <conditionalFormatting sqref="F3">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -2708,35 +3019,63 @@
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="H7" r:id="rId1" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H9" r:id="rId2" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H10" r:id="rId3" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H11" r:id="rId4" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H12" r:id="rId5" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H13" r:id="rId6" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H14" r:id="rId7" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H15" r:id="rId8" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H16" r:id="rId9" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H17" r:id="rId10" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H18" r:id="rId11" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H19" r:id="rId12" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H23" r:id="rId13" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H24" r:id="rId14" display="AliExpress search: M5 washer"/>
-    <hyperlink ref="H25" r:id="rId15" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H26" r:id="rId16" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H27" r:id="rId17" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H28" r:id="rId18" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H29" r:id="rId19" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H30" r:id="rId20" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H31" r:id="rId21" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H32" r:id="rId22" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H33" r:id="rId23" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H34" r:id="rId24" display="Bunnings search: 3 mm nails"/>
-    <hyperlink ref="H38" r:id="rId25" display="AliExpress search: 2.2k resistor"/>
-    <hyperlink ref="H44" r:id="rId26" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H45" r:id="rId27" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H46" r:id="rId28" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H47" r:id="rId29" display="AliExpress – DAZ's link"/>
-    <hyperlink ref="H48" r:id="rId30" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="I7" r:id="rId2" display="AliExpress search: MKS XDrive Mini"/>
+    <hyperlink ref="H9" r:id="rId3" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="I9" r:id="rId4" display="AliExpress search: E6B2-CWZ6C"/>
+    <hyperlink ref="H10" r:id="rId5" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="I10" r:id="rId6" display="AliExpress search: 13&quot; flat wheel"/>
+    <hyperlink ref="H11" r:id="rId7" display="AliExpress search: GT2 20T 6 mm bore"/>
+    <hyperlink ref="I11" r:id="rId8" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H12" r:id="rId9" display="AliExpress search: GT2 belt 212 mm"/>
+    <hyperlink ref="I12" r:id="rId10" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H13" r:id="rId11" display="AliExpress search: GT2 idler 20T 5 mm"/>
+    <hyperlink ref="I13" r:id="rId12" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H14" r:id="rId13" display="AliExpress search: 24V 10A power supply"/>
+    <hyperlink ref="I14" r:id="rId14" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H15" r:id="rId15" display="AliExpress search: XT60 pair"/>
+    <hyperlink ref="I15" r:id="rId16" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H16" r:id="rId17" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="I16" r:id="rId18" display="AliExpress search: 16 mm cross clamp"/>
+    <hyperlink ref="H17" r:id="rId19" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="I17" r:id="rId20" display="AliExpress search: 16 mm aluminium tube"/>
+    <hyperlink ref="H18" r:id="rId21" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="I18" r:id="rId22" display="AliExpress search: Arca-Swiss clamp"/>
+    <hyperlink ref="H19" r:id="rId23" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="I19" r:id="rId24" display="AliExpress search: Arca plate 100 mm"/>
+    <hyperlink ref="H23" r:id="rId25" display="AliExpress search: M5 nut"/>
+    <hyperlink ref="I23" r:id="rId26" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H24" r:id="rId27" display="AliExpress search: M5 washer"/>
+    <hyperlink ref="H25" r:id="rId28" display="AliExpress search: M5x20 socket head"/>
+    <hyperlink ref="I25" r:id="rId29" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H26" r:id="rId30" display="AliExpress search: M5x25 socket head"/>
+    <hyperlink ref="I26" r:id="rId31" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H27" r:id="rId32" display="AliExpress search: M5x40 socket head"/>
+    <hyperlink ref="I27" r:id="rId33" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H28" r:id="rId34" display="AliExpress search: M3x10 socket head"/>
+    <hyperlink ref="I28" r:id="rId35" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H29" r:id="rId36" display="AliExpress search: M3x12 self-tapping"/>
+    <hyperlink ref="I29" r:id="rId37" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H30" r:id="rId38" display="AliExpress search: M2.5x6 self-tapping"/>
+    <hyperlink ref="I30" r:id="rId39" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H31" r:id="rId40" display="AliExpress search: M6 nut"/>
+    <hyperlink ref="I31" r:id="rId41" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H32" r:id="rId42" display="AliExpress search: M6x30 countersunk"/>
+    <hyperlink ref="I32" r:id="rId43" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H33" r:id="rId44" display="AliExpress search: M6x45 countersunk"/>
+    <hyperlink ref="I33" r:id="rId45" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="H34" r:id="rId46" display="Bunnings search: 3 mm nails"/>
+    <hyperlink ref="H38" r:id="rId47" display="AliExpress search: 2.2k resistors"/>
+    <hyperlink ref="I38" r:id="rId48" display="AliExpress search: resistor kit"/>
+    <hyperlink ref="H44" r:id="rId49" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="I44" r:id="rId50" display="AliExpress search: wireless zero-delay encoder"/>
+    <hyperlink ref="H45" r:id="rId51" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="I45" r:id="rId52" display="AliExpress search: 16 mm push button"/>
+    <hyperlink ref="H46" r:id="rId53" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="I46" r:id="rId54" display="AliExpress search: 30×10×4 magnets"/>
+    <hyperlink ref="H47" r:id="rId55" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="I47" r:id="rId56" display="AliExpress search: 2 × AA holder"/>
+    <hyperlink ref="H48" r:id="rId57" display="AliExpress – DAZ's link"/>
+    <hyperlink ref="I48" r:id="rId58" display="AliExpress search: KW11-3Z roller switch"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>